<commit_message>
ongoing 1D implementation excel
</commit_message>
<xml_diff>
--- a/pNet/MTGHP-core/master.xlsx
+++ b/pNet/MTGHP-core/master.xlsx
@@ -8,34 +8,39 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\0_Python\pyHydraulics\pNet\MTGHP-core\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B700D754-0A2A-43E8-9125-41C8264F25FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6CD2E1-B5EE-4F8D-B044-C86DA189FA27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
   <si>
     <t>SN</t>
   </si>
   <si>
-    <t>From</t>
-  </si>
-  <si>
-    <t>To</t>
-  </si>
-  <si>
     <t>Inlet</t>
   </si>
   <si>
@@ -64,6 +69,39 @@
   </si>
   <si>
     <t>Channel</t>
+  </si>
+  <si>
+    <t>drain</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Upstream BC</t>
+  </si>
+  <si>
+    <t>Upstream BC Value</t>
+  </si>
+  <si>
+    <t>Upstream</t>
+  </si>
+  <si>
+    <t>Known WS</t>
+  </si>
+  <si>
+    <t>Downstream</t>
+  </si>
+  <si>
+    <t>Downstream BC</t>
+  </si>
+  <si>
+    <t>Downstream BC Value</t>
+  </si>
+  <si>
+    <t>Spill End</t>
+  </si>
+  <si>
+    <t>Spill Zero</t>
   </si>
 </sst>
 </file>
@@ -384,30 +422,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.81640625" customWidth="1"/>
-    <col min="2" max="2" width="9.81640625" customWidth="1"/>
-    <col min="3" max="3" width="11.90625" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" customWidth="1"/>
+    <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" customWidth="1"/>
+    <col min="4" max="4" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.1796875" customWidth="1"/>
+    <col min="7" max="7" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -415,66 +469,107 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+      <c r="E2">
+        <v>637</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+      <c r="F4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5">
+        <v>635.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B7" t="s">
         <v>11</v>
       </c>
-      <c r="D6" t="s">
-        <v>9</v>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7">
+        <v>625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TURFM and pNET in parallel
</commit_message>
<xml_diff>
--- a/pNet/MTGHP-core/master.xlsx
+++ b/pNet/MTGHP-core/master.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\0_Python\pyHydraulics\pNet\MTGHP-core\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6CD2E1-B5EE-4F8D-B044-C86DA189FA27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B0EEA8A-128C-481C-AEFE-F017CBA67BA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029" iterate="1" iterateCount="200"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -74,34 +74,34 @@
     <t>drain</t>
   </si>
   <si>
+    <t>Upstream BC</t>
+  </si>
+  <si>
+    <t>Upstream BC Value</t>
+  </si>
+  <si>
+    <t>Upstream</t>
+  </si>
+  <si>
+    <t>Known WS</t>
+  </si>
+  <si>
+    <t>Downstream</t>
+  </si>
+  <si>
+    <t>Downstream BC</t>
+  </si>
+  <si>
+    <t>Downstream BC Value</t>
+  </si>
+  <si>
+    <t>Spill End</t>
+  </si>
+  <si>
+    <t>Spill Zero</t>
+  </si>
+  <si>
     <t>None</t>
-  </si>
-  <si>
-    <t>Upstream BC</t>
-  </si>
-  <si>
-    <t>Upstream BC Value</t>
-  </si>
-  <si>
-    <t>Upstream</t>
-  </si>
-  <si>
-    <t>Known WS</t>
-  </si>
-  <si>
-    <t>Downstream</t>
-  </si>
-  <si>
-    <t>Downstream BC</t>
-  </si>
-  <si>
-    <t>Downstream BC Value</t>
-  </si>
-  <si>
-    <t>Spill End</t>
-  </si>
-  <si>
-    <t>Spill Zero</t>
   </si>
 </sst>
 </file>
@@ -443,22 +443,22 @@
         <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" t="s">
-        <v>14</v>
-      </c>
       <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
         <v>17</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>18</v>
-      </c>
-      <c r="H1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -472,7 +472,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2">
         <v>637</v>
@@ -509,7 +509,7 @@
         <v>7</v>
       </c>
       <c r="G4" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -526,10 +526,7 @@
         <v>7</v>
       </c>
       <c r="G5" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5">
-        <v>635.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -546,7 +543,7 @@
         <v>7</v>
       </c>
       <c r="G6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -560,13 +557,13 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F7" t="s">
         <v>7</v>
       </c>
       <c r="G7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H7">
         <v>625</v>

</xml_diff>